<commit_message>
Upload AI Audit Log
</commit_message>
<xml_diff>
--- a/AI_Audit_Log.xlsx
+++ b/AI_Audit_Log.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_IT\Semester\SU26\SE20C02_LAB211_SU26\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DB4BAFD-22E4-4A56-8BB6-7291655F4E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView windowWidth="23040" windowHeight="11148"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -20,9 +14,6 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -34,35 +25,14 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>Ví dụ: Abstraction</t>
-  </si>
-  <si>
-    <t>“Tôi cần quản lý thông tin sinh viên cho app quản lý điểm. Hãy liệt kê các thuộc tính cần thiết."</t>
-  </si>
-  <si>
-    <t>Ví dụ: Process/Algorithm</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition</t>
-  </si>
-  <si>
-    <t>“So sánh các giải thuật CPU scheduling: FCFS, SJF, Round Robin, Priority. Giải thuật nào tốt nhất?”</t>
-  </si>
-  <si>
-    <t>Ví dụ: Pattern Recognition + Literature Review</t>
-  </si>
-  <si>
-    <t>“Tóm tắt 5 bài báo gần đây nhất về anomaly detection trong IoT sensor data.”</t>
+    <t>STT</t>
   </si>
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
@@ -73,39 +43,22 @@
   <si>
     <t>Phản hồi của AI &amp; Quyết định của người học (Reflection)</t>
   </si>
-  <si>
-    <t>STT</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI liệt kê 20 thuộc tính.
-Quyết định: Tôi chỉ chọn 10 thuộc tính liên quan đến chức năng đang được yêu cầu từ ứng dụng (CCCD, địa chỉ...) và lược bỏ 10 thuộc tính học thuật vì phù hợp với yêu cầu của ứng dụng</t>
-  </si>
-  <si>
-    <t>"Viết hàm C sắp xếp mảng sinh viên theo điểm số bằng Selection Sort."</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI cung cấp code mẫu.
-Kiểm chứng: Tôi nhận thấy code AI chưa xử lý trường hợp mảng rỗng (Oversimplification). Tôi đã yêu cầu AI tối ưu lại và tự tay bổ sung điều kiện kiểm tra lỗi.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI response Round Robin là “tốt nhất” vì cân bằng giữa throughput và fairness.
-Kiểm chứng: AI đưa kết luận sai – không có giải thuật “tốt nhất” tuyệt đối (Hallucination). Mỗi giải thuật phù hợp với tình huống/context khác nhau.</t>
-  </si>
-  <si>
-    <t>Phản hồi: AI tóm tắt 5 papers với tên tác giả, năm xuất bản và tóm tắt nội dung.
-Kiểm chứng: Tìm trên Google Scholar: 2/5 papers AI nêu là không tồn tại (fabrication). Tôi đã thay bằng 2 papers mà tôi đã tìm kiếm trên research gates và đã kiểm chứng trên google scholar.</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
     </font>
@@ -114,19 +67,356 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -136,25 +426,270 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -165,26 +700,67 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -233,7 +809,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -266,26 +842,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -318,23 +877,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -496,125 +1038,103 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBDDC7E-59F2-4CBB-B3D2-F6FB78F9E873}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelRow="4" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="20.9296875" customWidth="1"/>
-    <col min="2" max="2" width="26.86328125" customWidth="1"/>
-    <col min="3" max="3" width="24.265625" customWidth="1"/>
+    <col min="1" max="1" width="20.9333333333333" customWidth="1"/>
+    <col min="2" max="2" width="26.8666666666667" customWidth="1"/>
+    <col min="3" max="3" width="24.2666666666667" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="5" t="s">
-        <v>10</v>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A2" s="2">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>0</v>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>11</v>
-      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="6"/>
     </row>
-    <row r="3" spans="1:5" ht="57" x14ac:dyDescent="0.45">
-      <c r="A3" s="2">
+    <row r="3" spans="1:5">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="6"/>
     </row>
-    <row r="4" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
-      <c r="A4" s="2">
+    <row r="4" spans="1:5">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="6"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E3EFE9-6FFB-49CC-BE69-0C0E36C6253E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>